<commit_message>
Atualização automática dos scripts ETL
</commit_message>
<xml_diff>
--- a/backend/objetos.xlsx
+++ b/backend/objetos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://leozed92-my.sharepoint.com/personal/leozed_leozed92_onmicrosoft_com/Documents/Aplicativos/App GAD SESAU/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="145" documentId="8_{C24DD8E0-50BB-40E4-B648-E8FAFBB74FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{595341F3-CC78-4EDD-A32A-3B9CE51153A8}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="8_{C24DD8E0-50BB-40E4-B648-E8FAFBB74FC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9A8B274-BF14-452D-997F-D3F652653A3D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" xr2:uid="{92D8D400-3915-4B7A-B5E9-ACA32B0E4BC3}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{92D8D400-3915-4B7A-B5E9-ACA32B0E4BC3}"/>
   </bookViews>
   <sheets>
     <sheet name="objetos" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="546">
   <si>
     <t>objeto</t>
   </si>
@@ -1627,6 +1627,57 @@
   </si>
   <si>
     <t>Construção de um Espaço de convivência - POC</t>
+  </si>
+  <si>
+    <t>0036.022430/2025-31</t>
+  </si>
+  <si>
+    <t>Monitor Multiparâmetro, equipamento permanente para atender as demandas das UTI 1 e UTI 2 do Hospital Regional de Cacoal - HRC.</t>
+  </si>
+  <si>
+    <t>Aquisição de Monitor Multiparâmetro, equipamento permanente para atender as demandas das UTI 1 e UTI 2 - HRC</t>
+  </si>
+  <si>
+    <t>0036.033047/2025-17</t>
+  </si>
+  <si>
+    <t>Contratação de curso II Fórum de Concessões e PPPs em Infraestrutura Social-Saúde, Educação, Segurança e Operações de transformação urbana, no dia 18 de setembro de 2025</t>
+  </si>
+  <si>
+    <t>0036.034011/2025-42</t>
+  </si>
+  <si>
+    <t>prestação de serviços técnicos de Engenharia Naval, visando à elaboração de Laudo Técnico e de Projeto Executivo de Recuperação Estrutural da embarcação Unidade de Saúde Social Fluvial Walter Bártolo, incluindo diagnóstico, especificações das intervenções necessárias, memorais descritivos, cronograma e demais documentos técnicos exigidos para a completa reabilitação e segurança operacional da embarcação.</t>
+  </si>
+  <si>
+    <t>0036.028208/2025-42</t>
+  </si>
+  <si>
+    <t>Emergencial - Limpeza, Conservação, Higienização e Desinfecção com Fornecimento de Materiais e Equipamentos (GRS4)</t>
+  </si>
+  <si>
+    <t>0035.001454/2025-67</t>
+  </si>
+  <si>
+    <t>Aquisição de ar condicionado com o objetivo de atender o Centro de Diálise de Ariquemes- CDA.</t>
+  </si>
+  <si>
+    <t>0046.000425/2025-59</t>
+  </si>
+  <si>
+    <t>Aquisição de condicionadores de ar (Central de Ar Condicionado), destinados ao atendimento das unidades de saúde (LABORATÓRIO CENTRAL DE SAÚDE PÚBLICA - LACEN/RO)</t>
+  </si>
+  <si>
+    <t>0050.007939/2025-76</t>
+  </si>
+  <si>
+    <t>JPII- Aquisição de Vídeo Laringoscópio Portátil.</t>
+  </si>
+  <si>
+    <t>0036.032294/2025-98</t>
+  </si>
+  <si>
+    <t>Aquisição de Materiais de Expediente - CLAP</t>
   </si>
 </sst>
 </file>
@@ -2008,7 +2059,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A2FF0CA-3C4D-4BFF-9AA5-A0CFD76751B1}">
-  <dimension ref="A1:C277"/>
+  <dimension ref="A1:C286"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
@@ -5026,6 +5077,87 @@
         <v>528</v>
       </c>
     </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>529</v>
+      </c>
+      <c r="B278" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>529</v>
+      </c>
+      <c r="B279" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>532</v>
+      </c>
+      <c r="B280" t="s">
+        <v>533</v>
+      </c>
+      <c r="C280" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>534</v>
+      </c>
+      <c r="B281" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>536</v>
+      </c>
+      <c r="B282" t="s">
+        <v>537</v>
+      </c>
+      <c r="C282" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>538</v>
+      </c>
+      <c r="B283" t="s">
+        <v>539</v>
+      </c>
+      <c r="C283" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
+        <v>540</v>
+      </c>
+      <c r="B284" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>542</v>
+      </c>
+      <c r="B285" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>544</v>
+      </c>
+      <c r="B286" t="s">
+        <v>545</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C249" xr:uid="{4A2FF0CA-3C4D-4BFF-9AA5-A0CFD76751B1}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>